<commit_message>
Further work on Schematics + parts
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Annie\code\hardware\ThermoBuzzer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D606D89E-8C49-4202-8384-99B5625D3371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F90D474-EF92-4B00-B0D2-C0F558AE7A7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3636" yWindow="1548" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>BOM</t>
   </si>
@@ -82,19 +82,40 @@
   </si>
   <si>
     <t>https://www.amazon.ca/ANALOG-DEVICES-TMP36-Temperature-Sensor/dp/B00JYQAIBM?source=ps-sl-shoppingads-lpcontext&amp;ref_=fplfs&amp;psc=1&amp;smid=AAEX2EKCSXB7D</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>NTC MF11</t>
+  </si>
+  <si>
+    <t>Battery</t>
+  </si>
+  <si>
+    <t>Arduino Nano (type)</t>
+  </si>
+  <si>
+    <t>Outlet with cabel?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF333333"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -117,8 +138,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -399,97 +423,115 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.88671875" customWidth="1"/>
-    <col min="2" max="2" width="20.109375" customWidth="1"/>
-    <col min="4" max="4" width="9.6640625" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" customWidth="1"/>
+    <col min="3" max="3" width="20.109375" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>6</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>7</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>9</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>10</v>
       </c>
-      <c r="C4">
+      <c r="B4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4">
         <v>1</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>11</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>12</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>1</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>1</v>
       </c>
-      <c r="C6">
+      <c r="D6">
         <v>1</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
-      <c r="C8">
+      <c r="D8">
         <v>1</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>17</v>
+      </c>
+      <c r="B9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finalize arduino + temperature
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Annie\code\hardware\ThermoBuzzer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F90D474-EF92-4B00-B0D2-C0F558AE7A7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A76CDC5D-D5C4-4E1E-B70E-46031212082A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3636" yWindow="1548" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
   <si>
     <t>BOM</t>
   </si>
@@ -60,9 +60,6 @@
     <t>Temperature Sensor</t>
   </si>
   <si>
-    <t>https://www.aliexpress.com/ssr/300000512/BundleDeals2?spm=a2g0o.productlist.main.11.4bad23b2W0Z283&amp;productIds=1005006982994037:12000038937173940&amp;pha_manifest=ssr&amp;_immersiveMode=true&amp;disableNav=YES&amp;sourceName=SEARCHProduct&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005006982994037%7C_p_origin_prod%3A1005007730203179&amp;pvid=fead97a0-7013-472f-8f48-f34087dd6ca8</t>
-  </si>
-  <si>
     <t>https://www.aliexpress.com/ssr/300000512/BundleDeals2?spm=a2g0o.productlist.main.12.4bad23b2W0Z283&amp;productIds=1005007345095808:12000040354473755&amp;pha_manifest=ssr&amp;_immersiveMode=true&amp;disableNav=YES&amp;sourceName=SEARCHProduct&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005007345095808%7C_p_origin_prod%3A1005006953448721&amp;pvid=fead97a0-7013-472f-8f48-f34087dd6ca8</t>
   </si>
   <si>
@@ -87,9 +84,6 @@
     <t>Type</t>
   </si>
   <si>
-    <t>NTC MF11</t>
-  </si>
-  <si>
     <t>Battery</t>
   </si>
   <si>
@@ -97,13 +91,31 @@
   </si>
   <si>
     <t>Outlet with cabel?</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005004904865598.html?spm=a2g0o.productlist.main.2.44c36f379bcEWK&amp;algo_pvid=37a4732e-0e3b-49dc-90f7-42ef2dc8c721&amp;algo_exp_id=37a4732e-0e3b-49dc-90f7-42ef2dc8c721-23&amp;pdp_ext_f=%7B%22order%22%3A%2213720%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21CAD%213.02%212.60%21%21%212.15%211.85%21%402101f70717742314163816448e5bdf%2112000030969396207%21sea%21CA%216218818596%21X%211%210%21n_tag%3A-29919%3Bd%3A26a99932%3Bm03_new_user%3A-29895&amp;curPageLogUid=BISAlr5fLDLJ&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005004904865598%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <t>NTC MF11, AHT20+BMP280</t>
+  </si>
+  <si>
+    <t>AHT20+BMP280 Temperature Humidity Air Pressure Module High-precision Digital Temperature Humidity and Air Pressure Sensor</t>
+  </si>
+  <si>
+    <t>5V</t>
+  </si>
+  <si>
+    <t>NA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00;[Red]\-&quot;$&quot;#,##0.00"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -116,6 +128,20 @@
       <color rgb="FF333333"/>
       <name val="Consolas"/>
       <family val="3"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="TT Norms Pro"/>
     </font>
   </fonts>
   <fills count="2">
@@ -135,16 +161,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -423,26 +454,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14.88671875" customWidth="1"/>
     <col min="2" max="2" width="15.6640625" customWidth="1"/>
     <col min="3" max="3" width="20.109375" customWidth="1"/>
-    <col min="5" max="5" width="9.6640625" customWidth="1"/>
+    <col min="6" max="6" width="9.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F1" s="1"/>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
         <v>5</v>
@@ -451,47 +483,59 @@
         <v>6</v>
       </c>
       <c r="E3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s">
         <v>7</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>9</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4">
+        <v>2.19</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G4" t="s">
+      <c r="I4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
         <v>12</v>
       </c>
-      <c r="H4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>13</v>
+      <c r="B5" t="s">
+        <v>25</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
-      <c r="E5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E5">
+        <v>3.99</v>
+      </c>
+      <c r="F5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -499,42 +543,57 @@
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
         <v>3</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>17</v>
-      </c>
       <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2">
+        <v>2.6</v>
+      </c>
+      <c r="F9" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9">
       <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" t="s">
         <v>21</v>
       </c>
-      <c r="B11" t="s">
-        <v>23</v>
-      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H4" r:id="rId1" display="https://www.aliexpress.com/ssr/300000512/BundleDeals2?spm=a2g0o.productlist.main.12.4bad23b2W0Z283&amp;productIds=1005007345095808:12000040354473755&amp;pha_manifest=ssr&amp;_immersiveMode=true&amp;disableNav=YES&amp;sourceName=SEARCHProduct&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005007345095808%7C_p_origin_prod%3A1005006953448721&amp;pvid=fead97a0-7013-472f-8f48-f34087dd6ca8" xr:uid="{8188D1EC-FE01-445E-8168-1909B737FBEE}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
april 4 schematic + footprints
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Annie\code\hardware\ThermoBuzzer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A76CDC5D-D5C4-4E1E-B70E-46031212082A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A5D29E5-89FA-4AE7-9A49-68AA36311231}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3636" yWindow="1548" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="29">
   <si>
     <t>BOM</t>
   </si>
@@ -90,9 +90,6 @@
     <t>Arduino Nano (type)</t>
   </si>
   <si>
-    <t>Outlet with cabel?</t>
-  </si>
-  <si>
     <t>https://www.aliexpress.com/item/1005004904865598.html?spm=a2g0o.productlist.main.2.44c36f379bcEWK&amp;algo_pvid=37a4732e-0e3b-49dc-90f7-42ef2dc8c721&amp;algo_exp_id=37a4732e-0e3b-49dc-90f7-42ef2dc8c721-23&amp;pdp_ext_f=%7B%22order%22%3A%2213720%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21CAD%213.02%212.60%21%21%212.15%211.85%21%402101f70717742314163816448e5bdf%2112000030969396207%21sea%21CA%216218818596%21X%211%210%21n_tag%3A-29919%3Bd%3A26a99932%3Bm03_new_user%3A-29895&amp;curPageLogUid=BISAlr5fLDLJ&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005004904865598%7C_p_origin_prod%3A</t>
   </si>
   <si>
@@ -106,6 +103,15 @@
   </si>
   <si>
     <t>NA</t>
+  </si>
+  <si>
+    <t>9v dc</t>
+  </si>
+  <si>
+    <t>Battery socket</t>
+  </si>
+  <si>
+    <t>https://www.amazon.ca/Duracell-Coppertop-Long-lasting-All-Purpose-Household/dp/B0014D0SL8/ref=asc_df_B0014D0SL8?mcid=c7225777934337b39c3f39a9df98d4c0&amp;tag=googleshopc0c-20&amp;linkCode=df0&amp;hvadid=706724917098&amp;hvpos=&amp;hvnetw=g&amp;hvrand=17738875034577000835&amp;hvpone=&amp;hvptwo=&amp;hvqmt=&amp;hvdev=c&amp;hvdvcmdl=&amp;hvlocint=&amp;hvlocphy=9000685&amp;hvtargid=pla-568057207376&amp;hvocijid=17738875034577000835-B0014D0SL8-&amp;hvexpln=0&amp;gad_source=4&amp;th=1</t>
   </si>
 </sst>
 </file>
@@ -454,7 +460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14.88671875" customWidth="1"/>
@@ -500,7 +506,7 @@
         <v>10</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -509,7 +515,7 @@
         <v>2.19</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>11</v>
@@ -523,7 +529,7 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -543,7 +549,7 @@
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F6" t="s">
         <v>14</v>
@@ -579,7 +585,7 @@
         <v>2.6</v>
       </c>
       <c r="F9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -587,7 +593,18 @@
         <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>26</v>
+      </c>
+      <c r="E11">
+        <v>9.98</v>
+      </c>
+      <c r="F11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>